<commit_message>
Refactor backend python(app) dengan memisahkan fungsi secara modular
</commit_message>
<xml_diff>
--- a/laporan/hasil_pengujian.xlsx
+++ b/laporan/hasil_pengujian.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uji Korektnas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uji Waktu" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Avalanche Effect" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entropi" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perbandingan Algoritma" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Uji Korektnas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Uji Waktu" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Avalanche Effect" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Entropi" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Perbandingan Algoritma" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2198,6 +2198,150 @@
         <v>1</v>
       </c>
       <c r="F73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>sample_data/README.md</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>682</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>aes-gcm</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>pbkdf2</t>
+        </is>
+      </c>
+      <c r="E74" t="b">
+        <v>1</v>
+      </c>
+      <c r="F74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>sample_data/README.md</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>682</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>aes-gcm</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>scrypt</t>
+        </is>
+      </c>
+      <c r="E75" t="b">
+        <v>1</v>
+      </c>
+      <c r="F75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>sample_data/README.md</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>682</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>aes-gcm</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>argon2</t>
+        </is>
+      </c>
+      <c r="E76" t="b">
+        <v>1</v>
+      </c>
+      <c r="F76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>sample_data/README.md</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>682</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>chacha20</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>pbkdf2</t>
+        </is>
+      </c>
+      <c r="E77" t="b">
+        <v>1</v>
+      </c>
+      <c r="F77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>sample_data/README.md</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>682</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>chacha20</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>scrypt</t>
+        </is>
+      </c>
+      <c r="E78" t="b">
+        <v>1</v>
+      </c>
+      <c r="F78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>sample_data/README.md</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>682</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>chacha20</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>argon2</t>
+        </is>
+      </c>
+      <c r="E79" t="b">
+        <v>1</v>
+      </c>
+      <c r="F79" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2280,16 +2424,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>165.967</v>
+        <v>626.7089999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>163.479</v>
+        <v>617.021</v>
       </c>
       <c r="F2" t="n">
-        <v>0.006</v>
+        <v>0.002</v>
       </c>
       <c r="G2" t="n">
-        <v>0.006</v>
+        <v>0.002</v>
       </c>
       <c r="H2" t="n">
         <v>5</v>
@@ -2310,16 +2454,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>155.009</v>
+        <v>659.924</v>
       </c>
       <c r="E3" t="n">
-        <v>151.693</v>
+        <v>675.961</v>
       </c>
       <c r="F3" t="n">
-        <v>0.006</v>
+        <v>0.001</v>
       </c>
       <c r="G3" t="n">
-        <v>0.006</v>
+        <v>0.001</v>
       </c>
       <c r="H3" t="n">
         <v>5</v>
@@ -2340,16 +2484,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>160.627</v>
+        <v>646.641</v>
       </c>
       <c r="E4" t="n">
-        <v>159.369</v>
+        <v>637.307</v>
       </c>
       <c r="F4" t="n">
-        <v>6.226</v>
+        <v>1.546</v>
       </c>
       <c r="G4" t="n">
-        <v>6.275</v>
+        <v>1.569</v>
       </c>
       <c r="H4" t="n">
         <v>5</v>
@@ -2370,16 +2514,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>156.384</v>
+        <v>642.359</v>
       </c>
       <c r="E5" t="n">
-        <v>149.77</v>
+        <v>644.575</v>
       </c>
       <c r="F5" t="n">
-        <v>6.395</v>
+        <v>1.557</v>
       </c>
       <c r="G5" t="n">
-        <v>6.677</v>
+        <v>1.551</v>
       </c>
       <c r="H5" t="n">
         <v>5</v>
@@ -2400,16 +2544,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>158.093</v>
+        <v>693.759</v>
       </c>
       <c r="E6" t="n">
-        <v>162.455</v>
+        <v>690.693</v>
       </c>
       <c r="F6" t="n">
-        <v>63.254</v>
+        <v>14.414</v>
       </c>
       <c r="G6" t="n">
-        <v>61.556</v>
+        <v>14.478</v>
       </c>
       <c r="H6" t="n">
         <v>5</v>
@@ -2430,16 +2574,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>155.166</v>
+        <v>687.511</v>
       </c>
       <c r="E7" t="n">
-        <v>150.23</v>
+        <v>677.148</v>
       </c>
       <c r="F7" t="n">
-        <v>64.447</v>
+        <v>14.545</v>
       </c>
       <c r="G7" t="n">
-        <v>66.565</v>
+        <v>14.768</v>
       </c>
       <c r="H7" t="n">
         <v>5</v>
@@ -2512,10 +2656,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>48.529</v>
+        <v>47.059</v>
       </c>
       <c r="E2" t="n">
-        <v>47.059</v>
+        <v>46.324</v>
       </c>
       <c r="F2" t="n">
         <v>50</v>
@@ -2534,10 +2678,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>51.471</v>
+        <v>55.147</v>
       </c>
       <c r="E3" t="n">
-        <v>49.265</v>
+        <v>47.794</v>
       </c>
       <c r="F3" t="n">
         <v>50</v>
@@ -2556,10 +2700,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>14.286</v>
+        <v>15.079</v>
       </c>
       <c r="E4" t="n">
-        <v>50</v>
+        <v>52.778</v>
       </c>
       <c r="F4" t="n">
         <v>50</v>
@@ -2578,10 +2722,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>13.294</v>
+        <v>12.698</v>
       </c>
       <c r="E5" t="n">
-        <v>50.595</v>
+        <v>47.222</v>
       </c>
       <c r="F5" t="n">
         <v>50</v>
@@ -2600,10 +2744,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3.217</v>
+        <v>2.941</v>
       </c>
       <c r="E6" t="n">
-        <v>49.678</v>
+        <v>47.426</v>
       </c>
       <c r="F6" t="n">
         <v>50</v>
@@ -2622,10 +2766,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2.482</v>
+        <v>2.619</v>
       </c>
       <c r="E7" t="n">
-        <v>49.081</v>
+        <v>50.368</v>
       </c>
       <c r="F7" t="n">
         <v>50</v>
@@ -2694,7 +2838,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7.9847</v>
+        <v>7.9866</v>
       </c>
     </row>
     <row r="4">
@@ -2709,7 +2853,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7.9849</v>
+        <v>7.9889</v>
       </c>
     </row>
   </sheetData>
@@ -2767,13 +2911,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6.226</v>
+        <v>1.546</v>
       </c>
       <c r="C2" t="n">
-        <v>6.275</v>
+        <v>1.569</v>
       </c>
       <c r="D2" t="n">
-        <v>22.011</v>
+        <v>21.693</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -2788,13 +2932,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6.395</v>
+        <v>1.557</v>
       </c>
       <c r="C3" t="n">
-        <v>6.677</v>
+        <v>1.551</v>
       </c>
       <c r="D3" t="n">
-        <v>22.416</v>
+        <v>23.488</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Menmbahkan tambahan UI, tes mandiri, dan tippy tooltip
Menerapkan pengukur kekuatan kata sandi, card algoritma interaktif,
breadcrumbs,
notifivation, pratinjau dropzone
</commit_message>
<xml_diff>
--- a/laporan/hasil_pengujian.xlsx
+++ b/laporan/hasil_pengujian.xlsx
@@ -2424,10 +2424,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>626.7089999999999</v>
+        <v>543.894</v>
       </c>
       <c r="E2" t="n">
-        <v>617.021</v>
+        <v>555.035</v>
       </c>
       <c r="F2" t="n">
         <v>0.002</v>
@@ -2454,10 +2454,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>659.924</v>
+        <v>673.2</v>
       </c>
       <c r="E3" t="n">
-        <v>675.961</v>
+        <v>663.552</v>
       </c>
       <c r="F3" t="n">
         <v>0.001</v>
@@ -2484,16 +2484,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>646.641</v>
+        <v>710.779</v>
       </c>
       <c r="E4" t="n">
-        <v>637.307</v>
+        <v>613.5170000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>1.546</v>
+        <v>1.407</v>
       </c>
       <c r="G4" t="n">
-        <v>1.569</v>
+        <v>1.63</v>
       </c>
       <c r="H4" t="n">
         <v>5</v>
@@ -2514,16 +2514,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>642.359</v>
+        <v>515.8200000000001</v>
       </c>
       <c r="E5" t="n">
-        <v>644.575</v>
+        <v>515.4450000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>1.557</v>
+        <v>1.939</v>
       </c>
       <c r="G5" t="n">
-        <v>1.551</v>
+        <v>1.94</v>
       </c>
       <c r="H5" t="n">
         <v>5</v>
@@ -2544,16 +2544,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>693.759</v>
+        <v>516.628</v>
       </c>
       <c r="E6" t="n">
-        <v>690.693</v>
+        <v>520.452</v>
       </c>
       <c r="F6" t="n">
-        <v>14.414</v>
+        <v>19.356</v>
       </c>
       <c r="G6" t="n">
-        <v>14.478</v>
+        <v>19.214</v>
       </c>
       <c r="H6" t="n">
         <v>5</v>
@@ -2574,16 +2574,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>687.511</v>
+        <v>547.869</v>
       </c>
       <c r="E7" t="n">
-        <v>677.148</v>
+        <v>533.813</v>
       </c>
       <c r="F7" t="n">
-        <v>14.545</v>
+        <v>18.253</v>
       </c>
       <c r="G7" t="n">
-        <v>14.768</v>
+        <v>18.733</v>
       </c>
       <c r="H7" t="n">
         <v>5</v>
@@ -2656,7 +2656,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>47.059</v>
+        <v>47.794</v>
       </c>
       <c r="E2" t="n">
         <v>46.324</v>
@@ -2678,10 +2678,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>55.147</v>
+        <v>50.735</v>
       </c>
       <c r="E3" t="n">
-        <v>47.794</v>
+        <v>48.529</v>
       </c>
       <c r="F3" t="n">
         <v>50</v>
@@ -2700,10 +2700,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>15.079</v>
+        <v>13.294</v>
       </c>
       <c r="E4" t="n">
-        <v>52.778</v>
+        <v>49.405</v>
       </c>
       <c r="F4" t="n">
         <v>50</v>
@@ -2722,10 +2722,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>12.698</v>
+        <v>14.087</v>
       </c>
       <c r="E5" t="n">
-        <v>47.222</v>
+        <v>51.786</v>
       </c>
       <c r="F5" t="n">
         <v>50</v>
@@ -2744,10 +2744,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2.941</v>
+        <v>2.711</v>
       </c>
       <c r="E6" t="n">
-        <v>47.426</v>
+        <v>50.46</v>
       </c>
       <c r="F6" t="n">
         <v>50</v>
@@ -2766,10 +2766,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2.619</v>
+        <v>2.711</v>
       </c>
       <c r="E7" t="n">
-        <v>50.368</v>
+        <v>49.54</v>
       </c>
       <c r="F7" t="n">
         <v>50</v>
@@ -2838,7 +2838,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7.9866</v>
+        <v>7.9872</v>
       </c>
     </row>
     <row r="4">
@@ -2853,7 +2853,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7.9889</v>
+        <v>7.987</v>
       </c>
     </row>
   </sheetData>
@@ -2911,13 +2911,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.546</v>
+        <v>1.407</v>
       </c>
       <c r="C2" t="n">
-        <v>1.569</v>
+        <v>1.63</v>
       </c>
       <c r="D2" t="n">
-        <v>21.693</v>
+        <v>21.266</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -2932,13 +2932,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.557</v>
+        <v>1.939</v>
       </c>
       <c r="C3" t="n">
-        <v>1.551</v>
+        <v>1.94</v>
       </c>
       <c r="D3" t="n">
-        <v>23.488</v>
+        <v>22.511</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Refaktor panel hybrid dan tambahkan fitur auto-reload untuk pengembangan
-Tambahkan persistensi sesi dan peningkatan status UI untuk enkripsi
hybrid RSA

-Implementasikan file watcher khusus pengembangan dan auto-refresh untuk
template dan aset statis

-Tingkatkan demo scenario runner dengan progress bar dan validasi
real-time
</commit_message>
<xml_diff>
--- a/laporan/hasil_pengujian.xlsx
+++ b/laporan/hasil_pengujian.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F79"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2198,150 +2198,6 @@
         <v>1</v>
       </c>
       <c r="F73" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>sample_data/README.md</t>
-        </is>
-      </c>
-      <c r="B74" t="n">
-        <v>682</v>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>aes-gcm</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>pbkdf2</t>
-        </is>
-      </c>
-      <c r="E74" t="b">
-        <v>1</v>
-      </c>
-      <c r="F74" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>sample_data/README.md</t>
-        </is>
-      </c>
-      <c r="B75" t="n">
-        <v>682</v>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>aes-gcm</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>scrypt</t>
-        </is>
-      </c>
-      <c r="E75" t="b">
-        <v>1</v>
-      </c>
-      <c r="F75" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>sample_data/README.md</t>
-        </is>
-      </c>
-      <c r="B76" t="n">
-        <v>682</v>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>aes-gcm</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>argon2</t>
-        </is>
-      </c>
-      <c r="E76" t="b">
-        <v>1</v>
-      </c>
-      <c r="F76" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>sample_data/README.md</t>
-        </is>
-      </c>
-      <c r="B77" t="n">
-        <v>682</v>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>chacha20</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>pbkdf2</t>
-        </is>
-      </c>
-      <c r="E77" t="b">
-        <v>1</v>
-      </c>
-      <c r="F77" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>sample_data/README.md</t>
-        </is>
-      </c>
-      <c r="B78" t="n">
-        <v>682</v>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>chacha20</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>scrypt</t>
-        </is>
-      </c>
-      <c r="E78" t="b">
-        <v>1</v>
-      </c>
-      <c r="F78" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>sample_data/README.md</t>
-        </is>
-      </c>
-      <c r="B79" t="n">
-        <v>682</v>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>chacha20</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>argon2</t>
-        </is>
-      </c>
-      <c r="E79" t="b">
-        <v>1</v>
-      </c>
-      <c r="F79" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2424,10 +2280,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>543.894</v>
+        <v>559.265</v>
       </c>
       <c r="E2" t="n">
-        <v>555.035</v>
+        <v>557.362</v>
       </c>
       <c r="F2" t="n">
         <v>0.002</v>
@@ -2454,16 +2310,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>673.2</v>
+        <v>561.501</v>
       </c>
       <c r="E3" t="n">
-        <v>663.552</v>
+        <v>562.526</v>
       </c>
       <c r="F3" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G3" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="H3" t="n">
         <v>5</v>
@@ -2484,16 +2340,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>710.779</v>
+        <v>559.419</v>
       </c>
       <c r="E4" t="n">
-        <v>613.5170000000001</v>
+        <v>556.071</v>
       </c>
       <c r="F4" t="n">
-        <v>1.407</v>
+        <v>1.788</v>
       </c>
       <c r="G4" t="n">
-        <v>1.63</v>
+        <v>1.798</v>
       </c>
       <c r="H4" t="n">
         <v>5</v>
@@ -2514,16 +2370,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>515.8200000000001</v>
+        <v>567.283</v>
       </c>
       <c r="E5" t="n">
-        <v>515.4450000000001</v>
+        <v>564.317</v>
       </c>
       <c r="F5" t="n">
-        <v>1.939</v>
+        <v>1.763</v>
       </c>
       <c r="G5" t="n">
-        <v>1.94</v>
+        <v>1.772</v>
       </c>
       <c r="H5" t="n">
         <v>5</v>
@@ -2544,16 +2400,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>516.628</v>
+        <v>566.765</v>
       </c>
       <c r="E6" t="n">
-        <v>520.452</v>
+        <v>568.085</v>
       </c>
       <c r="F6" t="n">
-        <v>19.356</v>
+        <v>17.644</v>
       </c>
       <c r="G6" t="n">
-        <v>19.214</v>
+        <v>17.603</v>
       </c>
       <c r="H6" t="n">
         <v>5</v>
@@ -2574,16 +2430,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>547.869</v>
+        <v>576.702</v>
       </c>
       <c r="E7" t="n">
-        <v>533.813</v>
+        <v>573.227</v>
       </c>
       <c r="F7" t="n">
-        <v>18.253</v>
+        <v>17.34</v>
       </c>
       <c r="G7" t="n">
-        <v>18.733</v>
+        <v>17.445</v>
       </c>
       <c r="H7" t="n">
         <v>5</v>
@@ -2656,10 +2512,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>47.794</v>
+        <v>43.382</v>
       </c>
       <c r="E2" t="n">
-        <v>46.324</v>
+        <v>49.265</v>
       </c>
       <c r="F2" t="n">
         <v>50</v>
@@ -2678,10 +2534,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>50.735</v>
+        <v>48.529</v>
       </c>
       <c r="E3" t="n">
-        <v>48.529</v>
+        <v>47.059</v>
       </c>
       <c r="F3" t="n">
         <v>50</v>
@@ -2700,10 +2556,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>13.294</v>
+        <v>12.302</v>
       </c>
       <c r="E4" t="n">
-        <v>49.405</v>
+        <v>50.595</v>
       </c>
       <c r="F4" t="n">
         <v>50</v>
@@ -2722,10 +2578,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>14.087</v>
+        <v>13.294</v>
       </c>
       <c r="E5" t="n">
-        <v>51.786</v>
+        <v>49.008</v>
       </c>
       <c r="F5" t="n">
         <v>50</v>
@@ -2744,10 +2600,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2.711</v>
+        <v>3.125</v>
       </c>
       <c r="E6" t="n">
-        <v>50.46</v>
+        <v>51.011</v>
       </c>
       <c r="F6" t="n">
         <v>50</v>
@@ -2766,10 +2622,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2.711</v>
+        <v>3.033</v>
       </c>
       <c r="E7" t="n">
-        <v>49.54</v>
+        <v>49.816</v>
       </c>
       <c r="F7" t="n">
         <v>50</v>
@@ -2838,7 +2694,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7.9872</v>
+        <v>7.989</v>
       </c>
     </row>
     <row r="4">
@@ -2853,7 +2709,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7.987</v>
+        <v>7.9872</v>
       </c>
     </row>
   </sheetData>
@@ -2911,13 +2767,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.407</v>
+        <v>1.788</v>
       </c>
       <c r="C2" t="n">
-        <v>1.63</v>
+        <v>1.798</v>
       </c>
       <c r="D2" t="n">
-        <v>21.266</v>
+        <v>19.603</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -2932,13 +2788,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.939</v>
+        <v>1.763</v>
       </c>
       <c r="C3" t="n">
-        <v>1.94</v>
+        <v>1.772</v>
       </c>
       <c r="D3" t="n">
-        <v>22.511</v>
+        <v>21.619</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>

</xml_diff>